<commit_message>
Enhance README with detailed application features and usage instructions; add main.spec for PyInstaller packaging
</commit_message>
<xml_diff>
--- a/load_cell_microseconds_20261029_181854.xlsx
+++ b/load_cell_microseconds_20261029_181854.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myerauedu-my.sharepoint.com/personal/niea_my_erau_edu/Documents/Documents/College Junior (2025-2026)/Project PIVOT/DAQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CF5F932-59D8-4473-95AD-307EE243C2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{7CF5F932-59D8-4473-95AD-307EE243C2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0165BFA-6EC2-4CE0-9B57-73C6FE576FAB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="24792" windowHeight="14856" xr2:uid="{86D66542-1210-455C-9565-210E91676DB7}"/>
   </bookViews>
@@ -652,32 +652,22 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="2"/>
           <c:order val="0"/>
           <c:spPr>
-            <a:ln w="38100" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent3"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
+            <c:symbol val="none"/>
           </c:marker>
           <c:xVal>
             <c:numRef>
@@ -7426,7 +7416,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-68AC-47B5-A303-88AD990CAAB7}"/>
@@ -7693,7 +7683,7 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -11019,26 +11009,16 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="38100" cap="rnd">
-              <a:noFill/>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
+            <c:symbol val="none"/>
           </c:marker>
           <c:xVal>
             <c:numRef>
@@ -17787,7 +17767,7 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-643D-4C38-98EC-EC5460B19516}"/>

</xml_diff>